<commit_message>
Mother Encore Web Site Act 2 Pré-Release 2
</commit_message>
<xml_diff>
--- a/src/assets/xlsx/translations.xlsx
+++ b/src/assets/xlsx/translations.xlsx
@@ -60,7 +60,7 @@
     <t>SITE_FOOTER_DISCLAIMER_1</t>
   </si>
   <si>
-    <t>Disclaimer: MOTHER: Encore is a free, unofficial fan game putting an alternative spin on MOTHER 1 and is not affiliated with Nintendo or Shigesato Itoi. This game offers a uniquely different experience from the original and should not be seen as a replacement for it. In other words, if you are playing MOTHER: Encore, you are not playing MOTHER 1.</t>
+    <t>Disclaimer: MOTHER: Encore is a free, unofficial fan game offering an alternative spin on MOTHER 1 and is not affiliated with Nintendo or Shigesato Itoi. This game provides a uniquely different experience from the original and should not be seen as a replacement for it. In other words, if you are playing MOTHER: Encore, you are not playing MOTHER 1.</t>
   </si>
   <si>
     <t>SITE_FOOTER_DISCLAIMER_2</t>
@@ -96,7 +96,7 @@
     <t>SITE_HOME_INTRO_2</t>
   </si>
   <si>
-    <t xml:space="preserve">Back in the year 1988, in a small rural town in America, a boy named Ninten woke up to the sight of many strange phenomena. Objects coming to life, animals going crazy, people vanishing without a trace, and a great shadowy cloud atop Mt Itoi... These are just a few of the many abnormal things happening all over America. Equipped with PSI powers, and following in his Great Grandfather's footsteps, will Ninten be able to uncover these many mysteries? </t>
+    <t xml:space="preserve">Back in the year 1988, in a small rural town in America, a boy named Ninten woke up to the sight of many strange phenomena. Objects coming to life, animals going crazy, people vanishing without a trace, and a great shadowy cloud atop Mt Itoi... these are just a few of the many bizarre things happening across the country. Equipped with PSI powers, and raring to follow in his great-grandfather's footsteps, will Ninten be able to uncover these many mysteries? </t>
   </si>
   <si>
     <t>SITE_HOME_INTRO_3</t>
@@ -120,7 +120,7 @@
     <t>SITE_HOME_NINTEN_1</t>
   </si>
   <si>
-    <t>This is you! A spirited young boy with a passion for baseball and uncovering mysteries. Ninten's favorite things to after a day at school is digging into some prime ribs, watching Star Wars on VHS, and trying to figure out what on Earth happened to his great-grandparents.</t>
+    <t>This is you! A spirited young boy with a passion for baseball and uncovering mysteries. Ninten's favorite things to do after a day at school are digging into some prime ribs, watching Star Wars on VHS, and trying to figure out what on Earth happened to his great-grandparents.</t>
   </si>
   <si>
     <t>SITE_HOME_NINTEN_2</t>
@@ -138,13 +138,13 @@
     <t>SITE_HOME_LLOYD_1</t>
   </si>
   <si>
-    <t>While he may look like a weakling, Lloyd's determined to prove his worth! He's got an array of inventions at his disposal, and he won't hesitate to use them. Even if he isn't the strongest, as long as you don't give up on him, he won't give up on you.</t>
+    <t>While he may look like a weakling, Lloyd's determined to prove his worth! He's got an array of inventions up his sleeve, and he won't hesitate to use them. Even if he isn't the strongest, as long as you don't give up on him, he won't give up on you.</t>
   </si>
   <si>
     <t>SITE_HOME_LLOYD_2</t>
   </si>
   <si>
-    <t>After years of dealing with bullies on his own, a certain friend is all he needs to unlock his courage.</t>
+    <t>After years of relentless bullying, a certain friend is all he needs to unlock his courage.</t>
   </si>
   <si>
     <t>SITE_HOME_ANA_TITLE</t>
@@ -156,13 +156,13 @@
     <t>SITE_HOME_ANA_1</t>
   </si>
   <si>
-    <t xml:space="preserve">She's a polite young girl from Snowman, whose docile personality was fostered by her town. Her favorite things to do are playing the piano and taking part in Bible studies. She's so beloved by everyone, some even consider her an angel. </t>
+    <t xml:space="preserve">A polite young girl whose docile personality was fostered by the community of Snowman. Ana's favorite things to do are playing the piano, singing to imported music records and taking part in Bible studies. She's so beloved by the little village, some even consider her an angel. </t>
   </si>
   <si>
     <t>SITE_HOME_ANA_2</t>
   </si>
   <si>
-    <t>Word on the wind says she's got mysterious PSI abilities, but it seems she doesn't like using them...</t>
+    <t>Word on the wind says she's got mysterious powers, but it seems she doesn't like using them...</t>
   </si>
   <si>
     <t>SITE_HOME_TEDDY_TITLE</t>
@@ -174,7 +174,7 @@
     <t>SITE_HOME_TEDDY_1</t>
   </si>
   <si>
-    <t>It's the notorious, tobacco chewing, knife-wielding leader of the BB Gang, Teddy! With years of crime and fighting experience, you'd be a fool to mess with him. He's just as threatening as he looks, but if he considers you a brother, he'll fight by your side until the bitter end.</t>
+    <t>Watch out! It's the notorious, tobacco-chewing, knife-wielding leader of the B.B. Gang, Teddy! With years of crime and fighting behind his back, you'd be a fool to mess with him. He's just as tough as he looks, but if he considers you a brother, he'll stick by your side until the bitter end.</t>
   </si>
   <si>
     <t>SITE_HOME_TEDDY_2</t>
@@ -198,13 +198,13 @@
     <t>SITE_ABOUT_OVERVIEW_P1</t>
   </si>
   <si>
-    <t>MOTHER: Encore is a brand new fan made entry in the MOTHER series that spins a whole new take on MOTHER 1 to create an original yet familiar experience. Every aspect of this game is made with love and respect for the original, analyzing every part of it as well as supplemental material such as the Encyclopedia in an attempt to create our own version of this classic game.</t>
+    <t>MOTHER: Encore is a brand new fan made entry in the MOTHER series that spins a whole new take on MOTHER 1 to create an original yet familiar experience. Every aspect of this game is made with love and respect for the original by analyzing all of its corners, as well as supplemental material such as the Encyclopedia in an attempt to create our own version of this classic game.</t>
   </si>
   <si>
     <t>SITE_ABOUT_OVERVIEW_P2</t>
   </si>
   <si>
-    <t xml:space="preserve">Originally beginning as “MOTHER 30th Anniversary edition” in RPG Maker VX Ace, the scope of the project expanded to the point of no longer being a remake. Now made entirely from the ground up using the Godot Engine, Encore aims to adapt the original game into a completely fresh and new experience for modern audiences. </t>
+    <t xml:space="preserve">Originally beginning as “MOTHER 30th Anniversary edition” in RPG Maker VX Ace, the scope of the project expanded to the point of no longer being just a remake. Now made entirely from the ground up using the Godot Engine, Encore aims to adapt the original game into a completely fresh and new experience for modern audiences. </t>
   </si>
   <si>
     <t>SITE_ABOUT_COMBAT_TITLE</t>
@@ -216,7 +216,7 @@
     <t>SITE_ABOUT_COMBAT_P1</t>
   </si>
   <si>
-    <t xml:space="preserve">Encore's battle system introduces brand new mechanics such as SP, Encores, and Adrenaline Rushes that bring a whole new angle on how to engage enemies! You'll have to consider all your options and rely on quick thinking in order to defeat this game's dangerous foes.  </t>
+    <t>Encore's battle system introduces brand new mechanics! With Skill Points, Encores, Adrenaline Rushes, and more, there are plenty of unique ways to engage enemies! You'll have to consider all your options and rely on quick thinking in order to defeat this game's dangerous foes.</t>
   </si>
   <si>
     <t>SITE_ABOUT_FIELD_SKILLS_TITLE</t>
@@ -313,7 +313,7 @@
     <t xml:space="preserve">While modeled after MOTHER 1, Encore is meant to be a new and original game that only shares certain surface level traits with the classic game. We're basically designing the game as if it was a fourth MOTHER game, while using MOTHER 1 as a template. In a way, Encore is closer to something like a Disney adaptation of a classic fairy tale than just a remake. That is to say, Encore is a completely different experience from MOTHER 1 and should not be seen as a replacement for it. </t>
   </si>
   <si>
-    <t>SITE_FAQ_A2_3</t>
+    <t>SITE_FAQ_A2_2</t>
   </si>
   <si>
     <t>We won't stop you if you play Encore and not MOTHER 1, but just know that if you are playing MOTHER: Encore, then you are not playing MOTHER 1. We just hope you appreciate the differences between the two games rather than simply compare which one is "better".</t>
@@ -1312,7 +1312,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{53C13B73-3BA1-44A8-A9E4-16000489D212}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AF658152-CECB-46F4-A024-422C2EC985CB}" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>

</xml_diff>